<commit_message>
Finalize backend-driven Excel formulas and cleanup legacy logic
- Added new functionality to the Excel editor class to properly handle rows with empty values when presenting dataframes.

- Introduced minor aesthetic adjustments to the debt planning section in the design-capital file.

- Completed the integration of all required backend formulas for design-capital using JSON-based definitions.

- Migrated all remaining FFSS and design-capital formulas into formulas_map.json, with formulas added in chronological order to reflect the underlying time structure.

- Effectively completed the transition to dynamic backend-driven calculations (initial results have been reviewed, but further validation is still required).

- Deleted the auxiliary rest_formulas.json file.

- Extended the ExcelFormulaProcessor class with additional logic and edge-case handling required to support the migrated formulas and ensure correct execution.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="1" state="visible" r:id="rId1"/>
@@ -121,7 +121,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -142,10 +142,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="1" xfId="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -494,8 +490,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.08984375" customWidth="1" min="2" max="2"/>
   </cols>
@@ -553,10 +549,10 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="2" ht="15.5" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -606,10 +602,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="15.5" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -659,10 +655,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" ht="15.5" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -712,10 +708,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="15.5" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -765,10 +761,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="15.5" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -818,10 +814,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="15.5" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -871,10 +867,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="15.5" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -887,71 +883,47 @@
           <t>years</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15.5" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1001,10 +973,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="15.5" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>GRID</t>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1054,573 +1026,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Off-Grid</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>2031</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>2032</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>2033</v>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="12" ht="15.5" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Growth CAPEX</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" ht="15.5" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Acc. Growth CAPEX</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="15.5" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Maintenance CAPEX</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="15.5" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Acc. Maintenance CAPEX</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="15.5" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Total CAPEX</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="15.5" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Acc. Total CAPEX</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" ht="15.5" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Total Depreciation</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.5" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Total Annual Depreciation</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="15.5" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>OFF-GRID</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>RAB</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Hoja1">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16.6328125" customWidth="1" min="2" max="2"/>
@@ -1674,7 +1092,7 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="2" ht="15.5" customHeight="1">
+    <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Growth CAPEX</t>
@@ -1722,7 +1140,7 @@
         <v>0.07967632839653764</v>
       </c>
     </row>
-    <row r="3" ht="15.5" customHeight="1">
+    <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Acc. Growth CAPEX</t>
@@ -1770,7 +1188,7 @@
         <v>1.531597401658293</v>
       </c>
     </row>
-    <row r="4" ht="15.5" customHeight="1">
+    <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Maintenance CAPEX</t>
@@ -1818,7 +1236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="15.5" customHeight="1">
+    <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Acc. Maintenance CAPEX</t>
@@ -1866,7 +1284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="15.5" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Total CAPEX</t>
@@ -1914,7 +1332,7 @@
         <v>0.07967632839653764</v>
       </c>
     </row>
-    <row r="7" ht="15.5" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Acc. Total CAPEX</t>
@@ -1962,7 +1380,7 @@
         <v>1.531597401658293</v>
       </c>
     </row>
-    <row r="8" ht="15.5" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Total Depreciation</t>
@@ -1976,41 +1394,63 @@
       <c r="C8" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="15.5" customHeight="1">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Total Annual Depreciation</t>
@@ -2058,7 +1498,7 @@
         <v>0.1021064934438862</v>
       </c>
     </row>
-    <row r="10" ht="15.5" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>RAB</t>
@@ -2079,34 +1519,34 @@
         <v>0.3962544287869533</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.5300403942390276</v>
+        <v>0.5259225440199846</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>0.6504849465450439</v>
+        <v>0.5634926581051729</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>0.7577214998364629</v>
+        <v>0.5114670710495095</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.8143128609143969</v>
+        <v>0.4222724666753693</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.8236373195592019</v>
+        <v>0.2898190396808248</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>0.8262185678426894</v>
+        <v>0.1738304013395598</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.8221240378684725</v>
+        <v>0.06447784362074217</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>0.8114204874191282</v>
+        <v>-0.001550165473407111</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>0.7952844545302826</v>
+        <v>-0.03256157880424315</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement electricity-specific formulas with grid divisions
- Completed backend formula implementation for electricity sector including:
  * Electricity & E-Cooking scenarios
  * Low access electricity scenarios
  * E-Cooking specific calculations

- Enhanced Excel formula processor to properly handle electricity's special case with multiple subdivisions

- Improved JSON formula expansion logic for complex electricity scenarios

- Added support for grid/off-grid differentiation in financial calculations

This represents the first iteration of electricity sector calculations. Further validation and refinement will be needed as part of the ongoing development process.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -490,8 +490,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="33.08984375" customWidth="1" min="2" max="2"/>
   </cols>
@@ -549,496 +549,1026 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="15.5" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.09441198237754599</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.1791091825492832</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0.1773180907237903</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0.1755449098165524</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0.1737894607183869</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>0.1720515661112031</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0.1300782577475552</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0.08872645212259944</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>0.08783918760137345</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>0.0869607957253597</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>0.08609118776810612</v>
+      </c>
+      <c r="O2" s="7" t="n">
+        <v>0.07967632839653764</v>
+      </c>
+    </row>
+    <row r="3" ht="15.5" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.09441198237754599</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.2735211649268292</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0.4508392556506195</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0.6263841654671719</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>0.8001736261855588</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>0.9722251922967619</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>1.102303450044317</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>1.191029902166916</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>1.27886908976829</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>1.36582988549365</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>1.451921073261756</v>
+      </c>
+      <c r="O3" s="7" t="n">
+        <v>1.531597401658293</v>
+      </c>
+    </row>
+    <row r="4" ht="15.5" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15.5" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15.5" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.09441198237754599</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.1791091825492832</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.1773180907237903</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0.1755449098165524</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0.1737894607183869</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.1720515661112031</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0.1300782577475552</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0.08872645212259944</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0.08783918760137345</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0.0869607957253597</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.08609118776810612</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>0.07967632839653764</v>
+      </c>
+    </row>
+    <row r="7" ht="15.5" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Acc. Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.09441198237754599</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.2735211649268292</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0.4508392556506195</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0.6263841654671719</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0.8001736261855588</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.9722251922967619</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>1.102303450044317</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>1.191029902166916</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>1.27886908976829</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>1.36582988549365</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>1.451921073261756</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>1.531597401658293</v>
+      </c>
+    </row>
+    <row r="8" ht="15.5" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Total Depreciation</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="15.5" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Total Annual Depreciation</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.006294132158503066</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.01823474432845528</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0.03005595037670796</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0.04175894436447813</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0.05334490841237059</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0.06481501281978412</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0.07348689666962113</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0.07940199347779443</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.085257939317886</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0.09105532569957665</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0.09679473821745038</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>0.1021064934438862</v>
+      </c>
+    </row>
+    <row r="10" ht="15.5" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>RAB</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.08811785021904292</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.2489922884398709</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0.3962544287869533</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0.5300403942390276</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>87.562367096326</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>84.5087292113966</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>81.41805843212745</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>78.29359692532019</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>75.17573362129767</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>72.06440253803203</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>68.99710762650474</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>65.96535300281259</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Off-Grid</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="12" ht="15.5" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Growth CAPEX</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="13" ht="15.5" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Acc. Growth CAPEX</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>3250</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>3900</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>4550</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>5850</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>7150</v>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>7800</v>
+      </c>
+    </row>
+    <row r="14" ht="15.5" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Maintenance CAPEX</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="15.5" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Acc. Maintenance CAPEX</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="15.5" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Total CAPEX</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="O16" s="7" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="17" ht="15.5" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Acc. Total CAPEX</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>3250</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>3900</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>4550</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>5850</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <v>7150</v>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>7800</v>
+      </c>
+    </row>
+    <row r="18" ht="15.5" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Total Depreciation</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="D18" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="15.5" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Total Annual Depreciation</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>38.23529411764706</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>76.47058823529412</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>114.7058823529412</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>152.9411764705882</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>191.1764705882353</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>229.4117647058823</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>267.6470588235294</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>305.8823529411765</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>344.1176470588235</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>382.3529411764706</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <v>420.5882352941176</v>
+      </c>
+      <c r="O19" s="7" t="n">
+        <v>458.8235294117647</v>
+      </c>
+    </row>
+    <row r="20" ht="15.5" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>OFF-GRID</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>RAB</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="7" t="n">
-        <v>0</v>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>611.7647058823529</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1185.294117647059</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>1720.588235294118</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>2217.64705882353</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>2142.420168067227</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1987.193277310924</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>1831.966386554622</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>1676.73949579832</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>1521.512605042016</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>1366.285714285714</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <v>1211.058823529412</v>
+      </c>
+      <c r="O20" s="7" t="n">
+        <v>1055.831932773109</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr codeName="Hoja1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16.6328125" customWidth="1" min="2" max="2"/>
@@ -1092,7 +1622,7 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="15.5" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Growth CAPEX</t>
@@ -1140,7 +1670,7 @@
         <v>0.07967632839653764</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15.5" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Acc. Growth CAPEX</t>
@@ -1188,7 +1718,7 @@
         <v>1.531597401658293</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="15.5" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Maintenance CAPEX</t>
@@ -1236,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="15.5" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Acc. Maintenance CAPEX</t>
@@ -1284,7 +1814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="15.5" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Total CAPEX</t>
@@ -1332,7 +1862,7 @@
         <v>0.07967632839653764</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="15.5" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Acc. Total CAPEX</t>
@@ -1380,7 +1910,7 @@
         <v>1.531597401658293</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="15.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Total Depreciation</t>
@@ -1394,63 +1924,41 @@
       <c r="C8" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="15.5" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Total Annual Depreciation</t>
@@ -1498,7 +2006,7 @@
         <v>0.1021064934438862</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="15.5" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>RAB</t>
@@ -1519,34 +2027,34 @@
         <v>0.3962544287869533</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.5259225440199846</v>
+        <v>0.5300403942390276</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>0.5634926581051729</v>
+        <v>0.646367096326001</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>0.5114670710495095</v>
+        <v>0.7547292113965919</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.4222724666753693</v>
+        <v>0.8140584321274437</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.2898190396808248</v>
+        <v>0.8275969253201745</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>0.1738304013395598</v>
+        <v>0.8264002879643122</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.06447784362074217</v>
+        <v>0.8204025380320098</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>-0.001550165473407111</v>
+        <v>0.7257742931713977</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>-0.03256157880424315</v>
+        <v>0.5426863361459109</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear formula cache between sheet processing
- Fixed critical bug where cached values were incorrectly reused across different sheets

- Now clears `previously_calculated` cache before processing each sheet to ensure data integrity

- Minor improvements to Excel cell editor for handling empty cells

- Fixed label matching for "vs. BAU" targets - now uses flexible matching to handle special symbols in Carbon Credits section
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Electricity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LPG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ethanol" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -1002,28 +1003,28 @@
         <v>0.5300403942390276</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>87.562367096326</v>
+        <v>0.6504849465450439</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>84.5087292113966</v>
+        <v>87.66960364961743</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>81.41805843212745</v>
+        <v>84.56532057247453</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>78.29359692532019</v>
+        <v>81.42738289077226</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>75.17573362129767</v>
+        <v>78.29617817360368</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>72.06440253803203</v>
+        <v>75.17163909132346</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>68.99710762650474</v>
+        <v>72.05369898758268</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>65.96535300281259</v>
+        <v>68.9746774614574</v>
       </c>
     </row>
     <row r="11">
@@ -1532,28 +1533,28 @@
         <v>2217.64705882353</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>2142.420168067227</v>
+        <v>2676.470588235295</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>1987.193277310924</v>
+        <v>2563.008403361345</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1831.966386554622</v>
+        <v>2369.546218487395</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1676.73949579832</v>
+        <v>2176.084033613445</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1521.512605042016</v>
+        <v>1982.621848739496</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>1366.285714285714</v>
+        <v>1789.159663865545</v>
       </c>
       <c r="N20" s="7" t="n">
-        <v>1211.058823529412</v>
+        <v>1595.697478991596</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>1055.831932773109</v>
+        <v>1402.235294117647</v>
       </c>
     </row>
   </sheetData>
@@ -1634,40 +1635,40 @@
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>0.09441198237754599</v>
+        <v>0.09</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>0.1791091825492832</v>
+        <v>0.18</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>0.1773180907237903</v>
+        <v>0.18</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>0.1755449098165524</v>
+        <v>0.18</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.1737894607183869</v>
+        <v>0.17</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>0.1720515661112031</v>
+        <v>0.17</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>0.1300782577475552</v>
+        <v>0.13</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>0.08872645212259944</v>
+        <v>0.09</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>0.08783918760137345</v>
+        <v>0.09</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>0.0869607957253597</v>
+        <v>0.09</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>0.08609118776810612</v>
+        <v>0.09</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>0.07967632839653764</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1">
@@ -1682,40 +1683,40 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>0.09441198237754599</v>
+        <v>0.09</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>0.2735211649268292</v>
+        <v>0.27</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.4508392556506195</v>
+        <v>0.45</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0.6263841654671719</v>
+        <v>0.63</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.8001736261855588</v>
+        <v>0.8</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.9722251922967619</v>
+        <v>0.9700000000000001</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1.102303450044317</v>
+        <v>1.1</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1.191029902166916</v>
+        <v>1.19</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1.27886908976829</v>
+        <v>1.28</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.36582988549365</v>
+        <v>1.37</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>1.451921073261756</v>
+        <v>1.46</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>1.531597401658293</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1">
@@ -1826,40 +1827,40 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.09441198237754599</v>
+        <v>0.09</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.1791091825492832</v>
+        <v>0.18</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.1773180907237903</v>
+        <v>0.18</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.1755449098165524</v>
+        <v>0.18</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>0.1737894607183869</v>
+        <v>0.17</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>0.1720515661112031</v>
+        <v>0.17</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0.1300782577475552</v>
+        <v>0.13</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>0.08872645212259944</v>
+        <v>0.09</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>0.08783918760137345</v>
+        <v>0.09</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.0869607957253597</v>
+        <v>0.09</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>0.08609118776810612</v>
+        <v>0.09</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>0.07967632839653764</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
@@ -1874,40 +1875,40 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>0.09441198237754599</v>
+        <v>0.09</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.2735211649268292</v>
+        <v>0.27</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.4508392556506195</v>
+        <v>0.45</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0.6263841654671719</v>
+        <v>0.63</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.8001736261855588</v>
+        <v>0.8</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.9722251922967619</v>
+        <v>0.9700000000000001</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1.102303450044317</v>
+        <v>1.1</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1.191029902166916</v>
+        <v>1.19</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1.27886908976829</v>
+        <v>1.28</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.36582988549365</v>
+        <v>1.37</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>1.451921073261756</v>
+        <v>1.46</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>1.531597401658293</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
@@ -1970,40 +1971,40 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.006294132158503066</v>
+        <v>0.006</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.01823474432845528</v>
+        <v>0.018</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03005595037670796</v>
+        <v>0.03</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.04175894436447813</v>
+        <v>0.042</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.05334490841237059</v>
+        <v>0.05333333333333334</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.06481501281978412</v>
+        <v>0.06466666666666668</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.07348689666962113</v>
+        <v>0.07333333333333333</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.07940199347779443</v>
+        <v>0.07933333333333334</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>0.085257939317886</v>
+        <v>0.08533333333333334</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>0.09105532569957665</v>
+        <v>0.09133333333333335</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>0.09679473821745038</v>
+        <v>0.09733333333333336</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>0.1021064934438862</v>
+        <v>0.1026666666666667</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -2018,43 +2019,541 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>0.08811785021904292</v>
+        <v>0.08399999999999999</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.2489922884398709</v>
+        <v>0.2501178502190429</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>0.3962544287869533</v>
+        <v>0.3989922884398709</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.5300403942390276</v>
+        <v>0.5342544287869533</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>0.646367096326001</v>
+        <v>0.6467070609056943</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>0.7547292113965919</v>
+        <v>0.7517004296593344</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.8140584321274437</v>
+        <v>0.8113958780632585</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.8275969253201745</v>
+        <v>0.8247250987941103</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>0.8264002879643122</v>
+        <v>0.8322635919868411</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.8204025380320098</v>
+        <v>0.8250669546309788</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>0.7257742931713977</v>
+        <v>0.8130692046986764</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>0.5426863361459109</v>
+        <v>0.703107626504731</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16.6328125" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D1" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E1" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F1" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G1" s="5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="H1" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="I1" s="5" t="n">
+        <v>2029</v>
+      </c>
+      <c r="J1" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="K1" s="5" t="n">
+        <v>2031</v>
+      </c>
+      <c r="L1" s="5" t="n">
+        <v>2032</v>
+      </c>
+      <c r="M1" s="5" t="n">
+        <v>2033</v>
+      </c>
+      <c r="N1" s="5" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Total CAPEX</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Acc. Total CAPEX</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Total Depreciation</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Total Annual Depreciation</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RAB</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>0.6646666666666666</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>0.5733333333333333</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.4759999999999999</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>0.3733333333333332</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Restructure Excel templates and backend for fuel-specific tariffs and upstream costs
- Split electricity demand, capex, opex, etc into "Electricity & E-Cooking" and "Electricity (Low access)"

- Updated Excel templates (technoeconomic, capex) to support new demand, capex, opex, etc categories

- Refactored backend formulas to use fuel-specific config lookups

- Implemented hierarchical config structure for tariffs and upstream costs per fuel type

- Detailed debugging and error handling for formula application process
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Electricity" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LPG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Electricity &amp; E-Cooking" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Electricity (Low access)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -566,40 +567,40 @@
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>257.2547513691348</v>
+        <v>2</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>324.6150491019822</v>
+        <v>324.62</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>321.3688986109623</v>
+        <v>321.37</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>318.1552096248527</v>
+        <v>318.16</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>314.9736575286042</v>
+        <v>314.97</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>311.8239209533182</v>
+        <v>311.82</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>382.0048802582858</v>
+        <v>382</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>451.1166131276156</v>
+        <v>451.12</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>446.6054469963394</v>
+        <v>446.61</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>442.139392526376</v>
+        <v>442.14</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>437.7179986011122</v>
+        <v>437.7179986011</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>290.7814303112916</v>
+        <v>290.78</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1">
@@ -619,40 +620,40 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>257.2547513691348</v>
+        <v>2</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>581.8698004711171</v>
+        <v>326.62</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>903.2386990820794</v>
+        <v>647.99</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>1221.393908706932</v>
+        <v>966.1500000000001</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1536.367566235536</v>
+        <v>1281.12</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1848.191487188854</v>
+        <v>1592.94</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>2230.19636744714</v>
+        <v>1974.94</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2681.312980574756</v>
+        <v>2426.06</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>3127.918427571095</v>
+        <v>2872.67</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>3570.057820097471</v>
+        <v>3314.81</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>4007.775818698583</v>
+        <v>3752.5279986011</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>4298.557249009875</v>
+        <v>4043.3079986011</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1">
@@ -778,40 +779,40 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>257.2547513691348</v>
+        <v>2</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>324.6150491019822</v>
+        <v>324.62</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>321.3688986109623</v>
+        <v>321.37</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>318.1552096248527</v>
+        <v>318.16</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>314.9736575286042</v>
+        <v>314.97</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>311.8239209533182</v>
+        <v>311.82</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>382.0048802582858</v>
+        <v>382</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>451.1166131276156</v>
+        <v>451.12</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>446.6054469963394</v>
+        <v>446.61</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>442.139392526376</v>
+        <v>442.14</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>437.7179986011122</v>
+        <v>437.7179986011</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>290.7814303112916</v>
+        <v>290.78</v>
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
@@ -831,40 +832,40 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>257.2547513691348</v>
+        <v>2</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>581.8698004711171</v>
+        <v>326.62</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>903.2386990820794</v>
+        <v>647.99</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>1221.393908706932</v>
+        <v>966.1500000000001</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1536.367566235536</v>
+        <v>1281.12</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1848.191487188854</v>
+        <v>1592.94</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>2230.19636744714</v>
+        <v>1974.94</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2681.312980574756</v>
+        <v>2426.06</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>3127.918427571095</v>
+        <v>2872.67</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>3570.057820097471</v>
+        <v>3314.81</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>4007.775818698583</v>
+        <v>3752.5279986011</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>4298.557249009875</v>
+        <v>4043.3079986011</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
@@ -937,40 +938,40 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>7.350135753403851</v>
+        <v>0.05714285714285714</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>16.62485144203191</v>
+        <v>9.332000000000001</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>25.8068199737737</v>
+        <v>18.514</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>34.89696882019806</v>
+        <v>27.60428571428572</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>43.89621617815818</v>
+        <v>36.60342857142857</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>52.80547106253869</v>
+        <v>45.51257142857143</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>63.71989621277544</v>
+        <v>56.42685714285714</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>76.60894230213587</v>
+        <v>69.316</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>89.36909793060272</v>
+        <v>82.07628571428572</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>102.0016520027849</v>
+        <v>94.70885714285714</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>114.5078805342452</v>
+        <v>107.2150856743172</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>122.8159214002821</v>
+        <v>115.5230856743171</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -990,40 +991,40 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>249.9046156157309</v>
+        <v>1.942857142857143</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>557.8948132756811</v>
+        <v>317.2308571428571</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>853.4568919128698</v>
+        <v>620.0868571428571</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1136.715132717525</v>
+        <v>1158.599714285714</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>1407.792574067971</v>
+        <v>1429.678044187159</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1416.994526193238</v>
+        <v>1688.687670418537</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1427.450187017019</v>
+        <v>2006.966891912871</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1506.543041345658</v>
+        <v>2381.473418431811</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>1580.654935572192</v>
+        <v>2738.718002639399</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>1649.835679297642</v>
+        <v>3078.860166815893</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>1801.046466176802</v>
+        <v>3402.074920931044</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>1647.622707965158</v>
+        <v>3570.035506082207</v>
       </c>
     </row>
     <row r="11">
@@ -1096,40 +1097,40 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>39.54004604566455</v>
+        <v>39.54</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>50.33243931157392</v>
+        <v>50.33</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>49.82911491845817</v>
+        <v>49.83</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>49.3308237692736</v>
+        <v>49.33</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>48.83751553158086</v>
+        <v>48.84</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>48.34914037626506</v>
+        <v>48.35</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>15.38261584720839</v>
+        <v>15.38</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>-17.09142019004943</v>
+        <v>-17.09</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>-16.92050598814893</v>
+        <v>-16.92</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>-16.75130092826744</v>
+        <v>-16.75</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>-16.58378791898477</v>
+        <v>-16.583787919</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>-1.667201492973772</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="13" ht="15.5" customHeight="1">
@@ -1149,40 +1150,40 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>39.54004604566455</v>
+        <v>39.54</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>89.87248535723847</v>
+        <v>89.87</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>139.7016002756966</v>
+        <v>139.7</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>189.0324240449702</v>
+        <v>189.03</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>237.8699395765511</v>
+        <v>237.87</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>286.2190799528162</v>
+        <v>286.22</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>301.6016958000246</v>
+        <v>301.6</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>284.5102756099752</v>
+        <v>284.51</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>267.5897696218262</v>
+        <v>267.59</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>250.8384686935588</v>
+        <v>250.84</v>
       </c>
       <c r="N13" s="7" t="n">
-        <v>234.254680774574</v>
+        <v>234.256212081</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>232.5874792816003</v>
+        <v>232.586212081</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
@@ -1308,40 +1309,40 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>39.54004604566455</v>
+        <v>39.54</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>50.33243931157392</v>
+        <v>50.33</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>49.82911491845817</v>
+        <v>49.83</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>49.3308237692736</v>
+        <v>49.33</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>48.83751553158086</v>
+        <v>48.84</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>48.34914037626506</v>
+        <v>48.35</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>15.38261584720839</v>
+        <v>15.38</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>-17.09142019004943</v>
+        <v>-17.09</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>-16.92050598814893</v>
+        <v>-16.92</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>-16.75130092826744</v>
+        <v>-16.75</v>
       </c>
       <c r="N16" s="7" t="n">
-        <v>-16.58378791898477</v>
+        <v>-16.583787919</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-1.667201492973772</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="17" ht="15.5" customHeight="1">
@@ -1361,40 +1362,40 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>39.54004604566455</v>
+        <v>39.54</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>89.87248535723847</v>
+        <v>89.87</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>139.7016002756966</v>
+        <v>139.7</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>189.0324240449702</v>
+        <v>189.03</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>237.8699395765511</v>
+        <v>237.87</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>286.2190799528162</v>
+        <v>286.22</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>301.6016958000246</v>
+        <v>301.6</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>284.5102756099752</v>
+        <v>284.51</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>267.5897696218262</v>
+        <v>267.59</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>250.8384686935588</v>
+        <v>250.84</v>
       </c>
       <c r="N17" s="7" t="n">
-        <v>234.254680774574</v>
+        <v>234.256212081</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>232.5874792816003</v>
+        <v>232.586212081</v>
       </c>
     </row>
     <row r="18" ht="15.5" customHeight="1">
@@ -1467,40 +1468,40 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>1.581601841826582</v>
+        <v>1.5816</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>3.594899414289539</v>
+        <v>3.5948</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>5.588064011027866</v>
+        <v>5.587999999999999</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>7.56129696179881</v>
+        <v>7.561199999999999</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>9.514797583062045</v>
+        <v>9.514799999999999</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>11.44876319811265</v>
+        <v>11.4488</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>12.06406783200098</v>
+        <v>12.064</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>11.38041102439901</v>
+        <v>11.3804</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>10.70359078487305</v>
+        <v>10.7036</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>10.03353874774235</v>
+        <v>10.0336</v>
       </c>
       <c r="N19" s="7" t="n">
-        <v>9.370187230982962</v>
+        <v>9.370248483239999</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>9.303499171264011</v>
+        <v>9.303448483239999</v>
       </c>
     </row>
     <row r="20" ht="15.5" customHeight="1">
@@ -1520,40 +1521,40 @@
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>37.95844420383797</v>
+        <v>37.9584</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>84.69598410112235</v>
+        <v>84.69359999999999</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>128.9370350085527</v>
+        <v>128.9356</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>170.7065618160275</v>
+        <v>170.7044</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>210.0292797645463</v>
+        <v>210.029644203838</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>820.7359186212135</v>
+        <v>246.9331841011223</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1350.846338503842</v>
+        <v>250.2482350085527</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1813.427574029022</v>
+        <v>221.7785618160275</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>2241.092773977938</v>
+        <v>194.1524797645463</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>2633.808745765174</v>
+        <v>167.3680569426987</v>
       </c>
       <c r="N20" s="7" t="n">
-        <v>2457.492208563104</v>
+        <v>141.4165685556661</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>2249.740775009709</v>
+        <v>130.4416888579777</v>
       </c>
     </row>
   </sheetData>
@@ -1562,6 +1563,1083 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="33.08984375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Grid</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E1" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F1" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G1" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H1" s="5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I1" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J1" s="5" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K1" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L1" s="5" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M1" s="5" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N1" s="5" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O1" s="5" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="2" ht="15.5" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>321.37</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>318.16</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>314.97</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>311.82</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>382</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>451.12</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>446.61</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>442.14</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>437.7179986011</v>
+      </c>
+      <c r="O2" s="7" t="n">
+        <v>290.78</v>
+      </c>
+    </row>
+    <row r="3" ht="15.5" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>325.37</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>643.53</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>958.5</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>1270.32</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>1652.32</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>2103.44</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>2550.05</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>2992.19</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>3429.9079986011</v>
+      </c>
+      <c r="O3" s="7" t="n">
+        <v>3720.6879986011</v>
+      </c>
+    </row>
+    <row r="4" ht="15.5" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15.5" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15.5" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>321.37</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>318.16</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>314.97</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>311.82</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>382</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>451.12</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>446.61</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>442.14</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>437.7179986011</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>290.78</v>
+      </c>
+    </row>
+    <row r="7" ht="15.5" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Acc. Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>325.37</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>643.53</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>958.5</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>1270.32</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>1652.32</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>2103.44</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>2550.05</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>2992.19</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>3429.9079986011</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>3720.6879986011</v>
+      </c>
+    </row>
+    <row r="8" ht="15.5" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Total Depreciation</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="15.5" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Total Annual Depreciation</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.05714285714285714</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.1142857142857143</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>9.296285714285714</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>18.38657142857143</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>27.38571428571429</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>36.29485714285714</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>47.20914285714286</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>60.09828571428572</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>72.85857142857144</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>85.49114285714286</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>97.99737138860286</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>106.3053713886029</v>
+      </c>
+    </row>
+    <row r="10" ht="15.5" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>RAB</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>1.942857142857143</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>3.828571428571429</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>315.9022857142857</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>615.6757142857143</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>903.2600000000001</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>1178.785142857143</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>1513.576</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>1904.597714285714</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>2526.310901330017</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>3189.063171926331</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>3512.268611372054</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>3680.236395619612</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Off-Grid</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>2031</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>2032</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>2033</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="12" ht="15.5" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>39.54</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>50.33</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>49.83</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>49.33</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>-17.09</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>-16.92</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>-16.75</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>-16.583787919</v>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="13" ht="15.5" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Growth CAPEX</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>39.54</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>89.87</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>139.7</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>189.03</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>237.87</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>286.22</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>301.6</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>284.51</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>267.59</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>250.84</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>234.256212081</v>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>232.586212081</v>
+      </c>
+    </row>
+    <row r="14" ht="15.5" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="15.5" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Acc. Maintenance CAPEX</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="15.5" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>39.54</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>50.33</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>49.83</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>49.33</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>-17.09</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>-16.92</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>-16.75</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>-16.583787919</v>
+      </c>
+      <c r="O16" s="7" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="17" ht="15.5" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Acc. Total CAPEX</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>39.54</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>89.87</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>139.7</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>189.03</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>237.87</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>286.22</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>301.6</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>284.51</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>267.59</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>250.84</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <v>234.256212081</v>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>232.586212081</v>
+      </c>
+    </row>
+    <row r="18" ht="15.5" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Total Depreciation</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="15.5" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Total Annual Depreciation</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>1.5816</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>3.5948</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>5.587999999999999</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>7.561199999999999</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>9.514799999999999</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>11.4488</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>12.064</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>11.3804</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>10.7036</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>10.0336</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <v>9.370248483239999</v>
+      </c>
+      <c r="O19" s="7" t="n">
+        <v>9.303448483239999</v>
+      </c>
+    </row>
+    <row r="20" ht="15.5" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>OFF-GRID</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>RAB</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>37.9584</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>84.69359999999999</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>128.9356</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>170.7044</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>210.0296</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>246.9308</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>250.2468</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>221.776444203838</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>194.1551841011223</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>167.3706350085527</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <v>141.4173254137875</v>
+      </c>
+      <c r="O20" s="7" t="n">
+        <v>130.4413948790663</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Hoja1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2033,25 +3111,25 @@
         <v>17.61428026283425</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>18.13440843089207</v>
+        <v>20.55392811964564</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>15.66908172438015</v>
+        <v>22.20616592147982</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>12.31376707487665</v>
+        <v>22.64726746976876</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>9.097205064264283</v>
+        <v>22.90394159947154</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>6.009421020252327</v>
+        <v>22.97699422218088</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>3.064995500387277</v>
+        <v>22.86722319037358</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>1.135595944586894</v>
+        <v>22.53036598800345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add input files and setup for country scenario
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -567,40 +567,40 @@
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>2</v>
+        <v>257.2547513691348</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>324.62</v>
+        <v>324.6150491019822</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>321.37</v>
+        <v>321.3688986109623</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>318.16</v>
+        <v>318.1552096248527</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>314.97</v>
+        <v>314.9736575286042</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>311.82</v>
+        <v>311.8239209533182</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>382</v>
+        <v>382.0048802582858</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>451.12</v>
+        <v>451.1166131276156</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>446.61</v>
+        <v>446.6054469963394</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>442.14</v>
+        <v>442.139392526376</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>437.7179986011</v>
+        <v>437.7179986011122</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>290.78</v>
+        <v>290.7814303112916</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1">
@@ -620,40 +620,40 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>2</v>
+        <v>257.2547513691348</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>326.62</v>
+        <v>581.8698004711171</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>647.99</v>
+        <v>903.2386990820794</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>966.1500000000001</v>
+        <v>1221.393908706932</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1281.12</v>
+        <v>1536.367566235536</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1592.94</v>
+        <v>1848.191487188854</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1974.94</v>
+        <v>2230.19636744714</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2426.06</v>
+        <v>2681.312980574756</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>2872.67</v>
+        <v>3127.918427571095</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>3314.81</v>
+        <v>3570.057820097471</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>3752.5279986011</v>
+        <v>4007.775818698583</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>4043.3079986011</v>
+        <v>4298.557249009875</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1">
@@ -779,40 +779,40 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2</v>
+        <v>257.2547513691348</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>324.62</v>
+        <v>324.6150491019822</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>321.37</v>
+        <v>321.3688986109623</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>318.16</v>
+        <v>318.1552096248527</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>314.97</v>
+        <v>314.9736575286042</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>311.82</v>
+        <v>311.8239209533182</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>382</v>
+        <v>382.0048802582858</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>451.12</v>
+        <v>451.1166131276156</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>446.61</v>
+        <v>446.6054469963394</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>442.14</v>
+        <v>442.139392526376</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>437.7179986011</v>
+        <v>437.7179986011122</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>290.78</v>
+        <v>290.7814303112916</v>
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
@@ -832,40 +832,40 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2</v>
+        <v>257.2547513691348</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>326.62</v>
+        <v>581.8698004711171</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>647.99</v>
+        <v>903.2386990820794</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>966.1500000000001</v>
+        <v>1221.393908706932</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1281.12</v>
+        <v>1536.367566235536</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1592.94</v>
+        <v>1848.191487188854</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1974.94</v>
+        <v>2230.19636744714</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2426.06</v>
+        <v>2681.312980574756</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>2872.67</v>
+        <v>3127.918427571095</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>3314.81</v>
+        <v>3570.057820097471</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>3752.5279986011</v>
+        <v>4007.775818698583</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>4043.3079986011</v>
+        <v>4298.557249009875</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
@@ -938,40 +938,40 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.05714285714285714</v>
+        <v>7.350135753403851</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>9.332000000000001</v>
+        <v>16.62485144203191</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>18.514</v>
+        <v>25.8068199737737</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>27.60428571428572</v>
+        <v>34.89696882019806</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>36.60342857142857</v>
+        <v>43.89621617815818</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>45.51257142857143</v>
+        <v>52.80547106253869</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>56.42685714285714</v>
+        <v>63.71989621277544</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>69.316</v>
+        <v>76.60894230213587</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>82.07628571428572</v>
+        <v>89.36909793060272</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>94.70885714285714</v>
+        <v>102.0016520027849</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>107.2150856743172</v>
+        <v>114.5078805342452</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>115.5230856743171</v>
+        <v>122.8159214002821</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -991,40 +991,40 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>1.942857142857143</v>
+        <v>249.9046156157309</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>317.2308571428571</v>
+        <v>557.8948132756811</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>620.0868571428571</v>
+        <v>853.4568919128698</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1158.599714285714</v>
+        <v>1136.715132717525</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>1429.678044187159</v>
+        <v>1407.792574067971</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1688.687670418537</v>
+        <v>1666.81102395875</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>2006.966891912871</v>
+        <v>1985.096008004261</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>2381.473418431811</v>
+        <v>2359.603678829741</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>2738.718002639399</v>
+        <v>2716.840027895478</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>3078.860166815893</v>
+        <v>3056.977768419069</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>3402.074920931044</v>
+        <v>3132.226128013061</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>3570.035506082207</v>
+        <v>3307.489439264119</v>
       </c>
     </row>
     <row r="11">
@@ -1533,28 +1533,28 @@
         <v>170.7044</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>210.029644203838</v>
+        <v>210.0296</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>246.9331841011223</v>
+        <v>246.9308</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>250.2482350085527</v>
+        <v>250.2468</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>221.7785618160275</v>
+        <v>221.7764</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>194.1524797645463</v>
+        <v>194.1528</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>167.3680569426987</v>
+        <v>167.3692</v>
       </c>
       <c r="N20" s="7" t="n">
-        <v>141.4165685556661</v>
+        <v>141.41516359776</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>130.4416888579777</v>
+        <v>130.44171511452</v>
       </c>
     </row>
   </sheetData>
@@ -1644,40 +1644,40 @@
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>2</v>
+        <v>214.8267851046716</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>2</v>
+        <v>248.0600347279134</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>321.37</v>
+        <v>245.5794343806341</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>318.16</v>
+        <v>243.1236400368279</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>314.97</v>
+        <v>240.6924036364595</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>311.82</v>
+        <v>238.285479600095</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>382</v>
+        <v>276.1328264022534</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>451.12</v>
+        <v>313.4000433206662</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>446.61</v>
+        <v>310.2660428874595</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>442.14</v>
+        <v>307.1633824585849</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>437.7179986011</v>
+        <v>304.091748633999</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>290.78</v>
+        <v>208.5872747268976</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1">
@@ -1697,40 +1697,40 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>2</v>
+        <v>214.8267851046716</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>4</v>
+        <v>462.886819832585</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>325.37</v>
+        <v>708.4662542132191</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>643.53</v>
+        <v>951.5898942500471</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>958.5</v>
+        <v>1192.282297886507</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1270.32</v>
+        <v>1430.567777486601</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1652.32</v>
+        <v>1706.700603888855</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2103.44</v>
+        <v>2020.100647209521</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>2550.05</v>
+        <v>2330.366690096981</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>2992.19</v>
+        <v>2637.530072555565</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>3429.9079986011</v>
+        <v>2941.621821189564</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>3720.6879986011</v>
+        <v>3150.209095916462</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1">
@@ -1856,40 +1856,40 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2</v>
+        <v>214.8267851046716</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2</v>
+        <v>248.0600347279134</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>321.37</v>
+        <v>245.5794343806341</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>318.16</v>
+        <v>243.1236400368279</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>314.97</v>
+        <v>240.6924036364595</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>311.82</v>
+        <v>238.285479600095</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>382</v>
+        <v>276.1328264022534</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>451.12</v>
+        <v>313.4000433206662</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>446.61</v>
+        <v>310.2660428874595</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>442.14</v>
+        <v>307.1633824585849</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>437.7179986011</v>
+        <v>304.091748633999</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>290.78</v>
+        <v>208.5872747268976</v>
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
@@ -1909,40 +1909,40 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2</v>
+        <v>214.8267851046716</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4</v>
+        <v>462.886819832585</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>325.37</v>
+        <v>708.4662542132191</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>643.53</v>
+        <v>951.5898942500471</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>958.5</v>
+        <v>1192.282297886507</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1270.32</v>
+        <v>1430.567777486601</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1652.32</v>
+        <v>1706.700603888855</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2103.44</v>
+        <v>2020.100647209521</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>2550.05</v>
+        <v>2330.366690096981</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>2992.19</v>
+        <v>2637.530072555565</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>3429.9079986011</v>
+        <v>2941.621821189564</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>3720.6879986011</v>
+        <v>3150.209095916462</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
@@ -2015,40 +2015,40 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.05714285714285714</v>
+        <v>6.13790814584776</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.1142857142857143</v>
+        <v>13.22533770950243</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>9.296285714285714</v>
+        <v>20.24189297752055</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>18.38657142857143</v>
+        <v>27.18828269285849</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>27.38571428571429</v>
+        <v>34.06520851104305</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>36.29485714285714</v>
+        <v>40.87336507104575</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>47.20914285714286</v>
+        <v>48.76287439682442</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>60.09828571428572</v>
+        <v>57.71716134884345</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>72.85857142857144</v>
+        <v>66.58190543134231</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>85.49114285714286</v>
+        <v>75.35800207301615</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>97.99737138860286</v>
+        <v>84.04633774827327</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>106.3053713886029</v>
+        <v>90.00597416904178</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -2068,40 +2068,40 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>1.942857142857143</v>
+        <v>208.6888769588238</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.828571428571429</v>
+        <v>443.5235739772348</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>315.9022857142857</v>
+        <v>668.8611153803483</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>615.6757142857143</v>
+        <v>678.0504529083511</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>903.2600000000001</v>
+        <v>651.7286653010709</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1178.785142857143</v>
+        <v>935.8769527127208</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1513.576</v>
+        <v>1247.084975945609</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1904.597714285714</v>
+        <v>1583.724948506301</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>2526.310901330017</v>
+        <v>1905.522114290512</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>3189.063171926331</v>
+        <v>2244.748399813509</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>3512.268611372054</v>
+        <v>2600.132643013126</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>3680.236395619612</v>
+        <v>2848.781234686293</v>
       </c>
     </row>
     <row r="11">
@@ -2619,19 +2619,19 @@
         <v>250.2468</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>221.776444203838</v>
+        <v>221.7764</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>194.1551841011223</v>
+        <v>194.1528</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>167.3706350085527</v>
+        <v>167.3692</v>
       </c>
       <c r="N20" s="7" t="n">
-        <v>141.4173254137875</v>
+        <v>141.41516359776</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>130.4413948790663</v>
+        <v>130.44171511452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve Manage Models workflow and BAU model handling
- Add horizontal separator between Manage Models and Outputs sections

- Remove year input when creating new models if BAU model already exists

- Inform user that the established BAU year range applies across all models

- Rename columns in Techno-Economic Inputs and CAPEX files from "Type - Inputs" to "System

- Adjust files created for BAU model (only CAPEX and Techno-Economic inputs; exclude Design Capital and Financial Statements)

- Optimize Manage Models: generate downloadable ZIP and template files only on button click, not on page load
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -11,7 +11,7 @@
     <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
 </file>
 
@@ -500,7 +500,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -1021,16 +1021,16 @@
         <v>3056.977768419069</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>3132.226128013061</v>
+        <v>3380.187886485936</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>3307.489439264119</v>
+        <v>3548.153395396945</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -2077,37 +2077,37 @@
         <v>668.8611153803483</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>678.0504529083511</v>
+        <v>884.7964727243178</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>651.7286653010709</v>
+        <v>1091.423667849734</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>935.8769527127208</v>
+        <v>1288.835782378783</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1247.084975945609</v>
+        <v>1516.205734384212</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1583.724948506301</v>
+        <v>1565.142596540069</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>1905.522114290512</v>
+        <v>1575.877751263489</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>2244.748399813509</v>
+        <v>1894.419304531659</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>2600.132643013126</v>
+        <v>2198.302786644844</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>2848.781234686293</v>
+        <v>2397.841177791569</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Restructure design-capital and update calculations
- Removed Grid/Off-Grid division structure from design-capital file

- Updated backend calculations to reflect new structure

- NOTE: Annual Cost of Service formula needs definition for combined Grid/Off-Grid scenarios (RAB, OPEX, Depreciation)

- Pending validation of calculation results
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -2098,10 +2098,10 @@
         <v>2247.378134197721</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>2260.677525267481</v>
+        <v>2467.423545083447</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>2146.30984309264</v>
+        <v>2379.258825825337</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Add iterative solver for circular financial calculations
- Implement convergence-based iteration (threshold: 0.01) to handle circular dependency between Annual Cost of Service and Taxes

- Update financial formulas: Annual Cost of Service, How much to be financed, Grants/Sub-debt financing, Equity - EoP

- Fix Financial Calculations table updates and sign conventions for Grants and Annual Cost of Service ratios

- Populate CO2 inputs

- Reset Upstream values to zero

- Clean up Spanish comments

- Restructure Annual Cost of Service position in sheet
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -3000,40 +3000,40 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>15</v>
+        <v>10.85629480038009</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0</v>
+        <v>30.20755940046954</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0</v>
+        <v>49.47365099229818</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0</v>
+        <v>68.65542130594864</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>0</v>
+        <v>87.75371355420268</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>0</v>
+        <v>106.7693625177143</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0</v>
+        <v>121.5605306920435</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>0</v>
+        <v>132.1562241375258</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>0</v>
+        <v>142.708999412179</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>0</v>
+        <v>153.2192856977115</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>0</v>
+        <v>163.6875078840145</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>0</v>
+        <v>173.9187208518351</v>
       </c>
     </row>
     <row r="9" ht="15.5" customHeight="1">
@@ -3048,40 +3048,40 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.178822834910969</v>
+        <v>0.2470771633403528</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.497573205873548</v>
+        <v>0.6874903662197818</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.8149206231511774</v>
+        <v>1.12596512641124</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.130879116280707</v>
+        <v>1.562520828341609</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>1.445462574503617</v>
+        <v>1.997176662593499</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.758684748168975</v>
+        <v>2.429951627843693</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>2.0023220731692</v>
+        <v>2.766582121230389</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>2.176852331844782</v>
+        <v>3.007728288340928</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>2.350675650526751</v>
+        <v>3.247897685743276</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.523799098615043</v>
+        <v>3.487100081134516</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>2.696229674815596</v>
+        <v>3.478267981194408</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>2.864756279990272</v>
+        <v>3.270705776201628</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -3096,40 +3096,40 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>2.503519688753565</v>
+        <v>2.435265360324181</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>6.787202047318703</v>
+        <v>17.63240252226354</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>10.73249268333197</v>
+        <v>41.126580786415</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>14.34099096399421</v>
+        <v>64.19792086738266</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>17.61428026283425</v>
+        <v>86.84886659697369</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>20.55392811964564</v>
+        <v>109.0818373686772</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>22.20616592147982</v>
+        <v>129.9699531393019</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>22.64726746976876</v>
+        <v>145.3792442784854</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>22.90394159947154</v>
+        <v>156.3397960336255</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>22.97699422218088</v>
+        <v>167.0733683023672</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>22.86722319037358</v>
+        <v>177.8282696803214</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>22.53036598800345</v>
+        <v>188.5081540506222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct calculations for Grants and Annual Cost of Service
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-CleanStep.xlsx
+++ b/backend/Rwanda/capex-fuels-CleanStep.xlsx
@@ -3000,40 +3000,40 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>10.85629480038009</v>
+        <v>-0.178822834910969</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>30.20755940046954</v>
+        <v>-0.497573205873548</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>49.47365099229818</v>
+        <v>-0.8149206231511774</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>68.65542130594864</v>
+        <v>-1.130879116280707</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>87.75371355420268</v>
+        <v>-1.445462574503617</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>106.7693625177143</v>
+        <v>-1.758684748168975</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>121.5605306920435</v>
+        <v>-2.0023220731692</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>132.1562241375258</v>
+        <v>-2.176852331844782</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>142.708999412179</v>
+        <v>-2.350675650526751</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>153.2192856977115</v>
+        <v>-2.523799098615043</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>163.6875078840145</v>
+        <v>-2.696229674815596</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>173.9187208518351</v>
+        <v>-2.864756279990272</v>
       </c>
     </row>
     <row r="9" ht="15.5" customHeight="1">
@@ -3048,40 +3048,40 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.2470771633403528</v>
+        <v>-14.99999999999999</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.6874903662197818</v>
+        <v>-41.7373882469716</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1.12596512641124</v>
+        <v>-68.35709406661381</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.562520828341609</v>
+        <v>-94.86029428319995</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>1.997176662593499</v>
+        <v>-121.2481539527606</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>2.429951627843693</v>
+        <v>-147.5218264807659</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>2.766582121230389</v>
+        <v>-167.9585893629945</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.007728288340928</v>
+        <v>-182.5985198922087</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>3.247897685743276</v>
+        <v>-197.1791509482349</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>3.487100081134516</v>
+        <v>-211.7010755258052</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>3.478267981194408</v>
+        <v>-226.1648806897039</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>3.270705776201628</v>
+        <v>-240.3012133279753</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -3096,40 +3096,40 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>2.435265360324181</v>
+        <v>17.68234252366453</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>17.63240252226354</v>
+        <v>49.02216350016385</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>41.126580786415</v>
+        <v>79.83625304466757</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>64.19792086738266</v>
+        <v>121.1773648384197</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>86.84886659697369</v>
+        <v>170.6337305647521</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>109.0818373686772</v>
+        <v>230.5365697269138</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>129.9699531393019</v>
+        <v>291.795751794866</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>145.3792442784854</v>
+        <v>345.8074788462422</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>156.3397960336255</v>
+        <v>399.4321417501947</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>167.0733683023672</v>
+        <v>448.4617549043493</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>177.8282696803214</v>
+        <v>492.9279752068693</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>188.5081540506222</v>
+        <v>532.5246864848719</v>
       </c>
     </row>
   </sheetData>

</xml_diff>